<commit_message>
Added new Gas Logic
Added piped Gas to block pricing, so now we do not have to split the Process LNG and Piped Gas anymore!
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2050.xlsx
+++ b/Input/urbs_intertemporal_2050/2050.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775CCAA8-8924-4C2C-BC27-0ABFAC09D007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB451F96-BD33-450C-BCD5-040B891B8075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" tabRatio="796" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="1" r:id="rId1"/>
@@ -2623,7 +2623,7 @@
         <v>23</v>
       </c>
       <c r="D5">
-        <v>8</v>
+        <v>20.52</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>24</v>
@@ -3266,13 +3266,13 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="A2:A12 B2:B3 C2:C12 P2:XFD4">
-    <cfRule type="expression" dxfId="13" priority="3">
+  <conditionalFormatting sqref="A4:C4 E4:F4">
+    <cfRule type="expression" dxfId="13" priority="14">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:F3 A4:C4 E4:F4">
-    <cfRule type="expression" dxfId="12" priority="14">
+  <conditionalFormatting sqref="A2:F3 P2:XFD4 A2:A12 C2:C12">
+    <cfRule type="expression" dxfId="12" priority="3">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3889,7 +3889,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
-  <conditionalFormatting sqref="A30:C31 E30:E31 A2:C19 E2:XFD19">
+  <conditionalFormatting sqref="A2:C19 E2:XFD19 A30:C31 E30:E31">
     <cfRule type="expression" dxfId="6" priority="5">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
@@ -3909,10 +3909,21 @@
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4:D5 D8:D13 D15:D19 D2">
+  <conditionalFormatting sqref="D2 D4:D5 D8:D13 D15:D19">
     <cfRule type="expression" dxfId="2" priority="13">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4">
+    <cfRule type="dataBar" priority="15">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D5 D8:D13 D15:D19 D2">
     <cfRule type="dataBar" priority="19">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -3930,16 +3941,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4">
-    <cfRule type="dataBar" priority="15">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D13 D15">
+  <conditionalFormatting sqref="D15 D13">
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="num" val="0"/>

</xml_diff>